<commit_message>
Rerun assemble_osc with 250606 dataset
Reannotated
</commit_message>
<xml_diff>
--- a/data/cell_annotations.xlsx
+++ b/data/cell_annotations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexis Weinreb\Projects\glia\osc_larva\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BFD067-ED3E-4DE2-BFC1-C49A353549F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6049568-61BC-4BD2-B7ED-FF7F660D9F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{2C4346A8-F236-4F7A-B473-746076003A96}"/>
+    <workbookView xWindow="-28920" yWindow="-4245" windowWidth="29040" windowHeight="15720" xr2:uid="{2C4346A8-F236-4F7A-B473-746076003A96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="164">
   <si>
     <t>putative_identity</t>
   </si>
@@ -179,9 +179,6 @@
     <t>PHsh</t>
   </si>
   <si>
-    <t>AM/PHso</t>
-  </si>
-  <si>
     <t>Could not separate AMso, PHso1, PHso2. Markers: grl-2, unc-53, lin-48, grl-12, F44A2.3, lin-44</t>
   </si>
   <si>
@@ -233,9 +230,6 @@
     <t>OLsh</t>
   </si>
   <si>
-    <t>Wormbase TEA shows enrichment for ILsh markers: R08A2.5, dyf-4, ttr-18, ttr-51, ttr-43, lipl-6, ZK856.7, ttr-15, gst-28, F33G12.6, nex-3, kcc-3, pros-1, bug-1, T19D12.6, BE10.4, M03E7.2, mam-8, spig-1, gegf-1, T23F2.3, txt-17, F59F5.7, nlp-16, hil-7, C11H1.7, gst-10, C25E10.5, lpr-1, fox-1, Y32G9B.1, lgc-27, H05C05.4</t>
-  </si>
-  <si>
     <t>glia_2</t>
   </si>
   <si>
@@ -245,9 +239,6 @@
     <t>CEPso</t>
   </si>
   <si>
-    <t>col-56, col-68</t>
-  </si>
-  <si>
     <t>ILso</t>
   </si>
   <si>
@@ -287,9 +278,6 @@
     <t>neuroblast_2</t>
   </si>
   <si>
-    <t>progenitor</t>
-  </si>
-  <si>
     <t>Matches neuroblasts in the Packer, CeNGEN L1, and Wormbase TEA data. Some specific genes: unc-42, zig-8, hlh-14, hlh-16, fezf-1</t>
   </si>
   <si>
@@ -510,6 +498,36 @@
   </si>
   <si>
     <t>PHC</t>
+  </si>
+  <si>
+    <t>AM_PHso</t>
+  </si>
+  <si>
+    <t>glia_socket_2</t>
+  </si>
+  <si>
+    <t>ADE_PDEso</t>
+  </si>
+  <si>
+    <t>Wormbase TEA shows enrichment for putative ILsh markers: dhsl-4, T23F2.3, R01H10.4, slt-1, C11H1.7, C25E10.5, lfi-1</t>
+  </si>
+  <si>
+    <t>Expresses genes reported as ADE/PDEso by wormglia.org: glam-3/F58F12.4, F18E9.4, efhd-1</t>
+  </si>
+  <si>
+    <t>Expresses col-56, col-68</t>
+  </si>
+  <si>
+    <t>glia_socket_3</t>
+  </si>
+  <si>
+    <t>OLso</t>
+  </si>
+  <si>
+    <t>Expresses genes reported as OLso markers by wormglia.org: C04F12.5, spig-13, cnc-10, lido-8, grd-16</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
 </sst>
 </file>
@@ -890,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F40488A-EE35-45C3-A1C0-867D2AA424CC}">
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -902,7 +920,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -914,40 +932,40 @@
         <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>154</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>44</v>
@@ -956,12 +974,12 @@
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
         <v>46</v>
@@ -970,40 +988,40 @@
         <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -1012,128 +1030,134 @@
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
         <v>62</v>
-      </c>
-      <c r="C13" t="s">
-        <v>63</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>155</v>
+      </c>
+      <c r="C15" t="s">
+        <v>156</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>160</v>
+      </c>
+      <c r="C16" t="s">
+        <v>161</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>38</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1141,13 +1165,13 @@
         <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1155,120 +1179,120 @@
         <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D18" t="s">
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>75</v>
+      </c>
+      <c r="C23" t="s">
+        <v>76</v>
       </c>
       <c r="D23" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="E24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B25" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D25" t="s">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="E25" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1276,100 +1300,100 @@
         <v>90</v>
       </c>
       <c r="B26" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>6</v>
+        <v>163</v>
       </c>
       <c r="E26" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B27" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>3</v>
+        <v>163</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>163</v>
       </c>
       <c r="E28" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D29" t="s">
-        <v>98</v>
+        <v>163</v>
       </c>
       <c r="E29" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" t="s">
         <v>94</v>
       </c>
-      <c r="B30" t="s">
-        <v>4</v>
-      </c>
-      <c r="D30" t="s">
-        <v>98</v>
-      </c>
       <c r="E30" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" t="s">
         <v>94</v>
       </c>
-      <c r="B31" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" t="s">
-        <v>13</v>
-      </c>
       <c r="E31" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1377,117 +1401,117 @@
         <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>2</v>
+        <v>163</v>
       </c>
       <c r="E33" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
         <v>2</v>
       </c>
       <c r="E34" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B35" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="D35" t="s">
         <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>25</v>
+      </c>
+      <c r="C36" t="s">
+        <v>24</v>
       </c>
       <c r="D36" t="s">
         <v>2</v>
       </c>
       <c r="E36" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>26</v>
+      </c>
+      <c r="C37" t="s">
+        <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B38" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="E38" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="D39" t="s">
-        <v>9</v>
+        <v>163</v>
       </c>
       <c r="E39" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D40" t="s">
-        <v>9</v>
+        <v>163</v>
       </c>
       <c r="E40" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1495,195 +1519,195 @@
         <v>90</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D41" t="s">
         <v>9</v>
       </c>
       <c r="E41" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B42" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D42" t="s">
         <v>9</v>
       </c>
       <c r="E42" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B43" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D43" t="s">
         <v>9</v>
       </c>
       <c r="E43" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B44" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D44" t="s">
         <v>9</v>
       </c>
       <c r="E44" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B45" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D45" t="s">
         <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D46" t="s">
         <v>9</v>
       </c>
       <c r="E46" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>101</v>
       </c>
       <c r="D47" t="s">
         <v>9</v>
       </c>
       <c r="E47" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B48" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D48" t="s">
         <v>9</v>
       </c>
       <c r="E48" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
       <c r="D49" t="s">
         <v>9</v>
       </c>
       <c r="E49" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D50" t="s">
         <v>9</v>
       </c>
       <c r="E50" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B51" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D51" t="s">
         <v>9</v>
       </c>
       <c r="E51" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B52" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D52" t="s">
         <v>9</v>
       </c>
       <c r="E52" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B53" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D53" t="s">
         <v>9</v>
       </c>
       <c r="E53" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B54" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D54" t="s">
         <v>9</v>
       </c>
       <c r="E54" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1691,503 +1715,503 @@
         <v>90</v>
       </c>
       <c r="B55" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D55" t="s">
         <v>9</v>
       </c>
       <c r="E55" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B56" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="D56" t="s">
         <v>9</v>
       </c>
       <c r="E56" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D57" t="s">
         <v>9</v>
       </c>
       <c r="E57" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B58" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D58" t="s">
         <v>9</v>
       </c>
       <c r="E58" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B59" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D59" t="s">
         <v>9</v>
       </c>
       <c r="E59" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B60" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D60" t="s">
         <v>9</v>
       </c>
       <c r="E60" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D61" t="s">
         <v>9</v>
       </c>
       <c r="E61" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B62" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D62" t="s">
         <v>9</v>
       </c>
       <c r="E62" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B63" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D63" t="s">
         <v>9</v>
       </c>
       <c r="E63" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B64" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D64" t="s">
         <v>9</v>
       </c>
       <c r="E64" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B65" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="D65" t="s">
         <v>9</v>
       </c>
       <c r="E65" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B66" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D66" t="s">
         <v>9</v>
       </c>
       <c r="E66" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B67" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D67" t="s">
         <v>9</v>
       </c>
       <c r="E67" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B68" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D68" t="s">
         <v>9</v>
       </c>
       <c r="E68" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="D69" t="s">
         <v>9</v>
       </c>
       <c r="E69" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B70" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D70" t="s">
         <v>9</v>
       </c>
       <c r="E70" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B71" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D71" t="s">
         <v>9</v>
       </c>
       <c r="E71" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B72" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D72" t="s">
         <v>9</v>
       </c>
       <c r="E72" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B73" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="D73" t="s">
         <v>9</v>
       </c>
       <c r="E73" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B74" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D74" t="s">
         <v>9</v>
       </c>
       <c r="E74" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D75" t="s">
         <v>9</v>
       </c>
       <c r="E75" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B76" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D76" t="s">
         <v>9</v>
       </c>
       <c r="E76" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B77" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="D77" t="s">
         <v>9</v>
       </c>
       <c r="E77" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B78" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D78" t="s">
         <v>9</v>
       </c>
       <c r="E78" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B79" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D79" t="s">
         <v>9</v>
       </c>
       <c r="E79" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B80" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D80" t="s">
         <v>9</v>
       </c>
       <c r="E80" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D81" t="s">
         <v>9</v>
       </c>
       <c r="E81" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B82" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D82" t="s">
         <v>9</v>
       </c>
       <c r="E82" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B83" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D83" t="s">
         <v>9</v>
       </c>
       <c r="E83" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D84" t="s">
         <v>9</v>
       </c>
       <c r="E84" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D85" t="s">
         <v>9</v>
       </c>
       <c r="E85" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D86" t="s">
         <v>9</v>
       </c>
       <c r="E86" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D87" t="s">
         <v>9</v>
       </c>
       <c r="E87" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D88" t="s">
         <v>9</v>
       </c>
       <c r="E88" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B89" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D89" t="s">
         <v>9</v>
       </c>
       <c r="E89" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B90" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D90" t="s">
         <v>9</v>
       </c>
       <c r="E90" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2195,102 +2219,130 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D91" t="s">
         <v>9</v>
       </c>
       <c r="E91" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B92" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D92" t="s">
         <v>9</v>
       </c>
       <c r="E92" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B93" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D93" t="s">
         <v>9</v>
       </c>
       <c r="E93" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B94" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D94" t="s">
         <v>9</v>
       </c>
       <c r="E94" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B95" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D95" t="s">
         <v>9</v>
       </c>
       <c r="E95" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B96" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D96" t="s">
         <v>9</v>
       </c>
       <c r="E96" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B97" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D97" t="s">
         <v>9</v>
       </c>
       <c r="E97" t="s">
-        <v>96</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>86</v>
+      </c>
+      <c r="B98" t="s">
+        <v>147</v>
+      </c>
+      <c r="D98" t="s">
+        <v>9</v>
+      </c>
+      <c r="E98" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>90</v>
+      </c>
+      <c r="B99" t="s">
+        <v>148</v>
+      </c>
+      <c r="D99" t="s">
+        <v>9</v>
+      </c>
+      <c r="E99" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A39:E97">
-    <sortCondition ref="B39:B97"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A41:E99">
+    <sortCondition ref="B41:B99"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add comment in cell annotation
</commit_message>
<xml_diff>
--- a/data/cell_annotations.xlsx
+++ b/data/cell_annotations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexis Weinreb\Projects\glia\osc_larva\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6049568-61BC-4BD2-B7ED-FF7F660D9F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC8192B3-0DE2-4E46-B042-D6B0D8B2C2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-4245" windowWidth="29040" windowHeight="15720" xr2:uid="{2C4346A8-F236-4F7A-B473-746076003A96}"/>
   </bookViews>
@@ -509,9 +509,6 @@
     <t>ADE_PDEso</t>
   </si>
   <si>
-    <t>Wormbase TEA shows enrichment for putative ILsh markers: dhsl-4, T23F2.3, R01H10.4, slt-1, C11H1.7, C25E10.5, lfi-1</t>
-  </si>
-  <si>
     <t>Expresses genes reported as ADE/PDEso by wormglia.org: glam-3/F58F12.4, F18E9.4, efhd-1</t>
   </si>
   <si>
@@ -528,6 +525,9 @@
   </si>
   <si>
     <t>other</t>
+  </si>
+  <si>
+    <t>Wormbase TEA shows enrichment for putative ILsh markers: dhsl-4, T23F2.3, R01H10.4, slt-1, C11H1.7, C25E10.5, lfi-1. High expression of sheath markers kcc-3, gegf-1, ttr-43</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1016,7 @@
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1106,7 +1106,7 @@
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1140,7 +1140,7 @@
         <v>5</v>
       </c>
       <c r="E15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1148,16 +1148,16 @@
         <v>86</v>
       </c>
       <c r="B16" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" t="s">
         <v>160</v>
-      </c>
-      <c r="C16" t="s">
-        <v>161</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1303,7 +1303,7 @@
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E26" t="s">
         <v>32</v>
@@ -1317,7 +1317,7 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E27" t="s">
         <v>15</v>
@@ -1334,7 +1334,7 @@
         <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -1348,7 +1348,7 @@
         <v>3</v>
       </c>
       <c r="D29" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E29" t="s">
         <v>28</v>
@@ -1404,7 +1404,7 @@
         <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E33" t="s">
         <v>36</v>
@@ -1494,7 +1494,7 @@
         <v>78</v>
       </c>
       <c r="D39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E39" t="s">
         <v>81</v>
@@ -1508,7 +1508,7 @@
         <v>79</v>
       </c>
       <c r="D40" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E40" t="s">
         <v>80</v>

</xml_diff>